<commit_message>
docs(deliverables): align spec/WBS with system diagrams (ERD·class·usecase)
- 추가된 docs/diagrams(ERD·클래스·유스케이스) 반영
- 데이터 명세 ERD 정합: member_refresh_tokens 정정, notices 추가, interest_regions 확정
- 누락 기능 보완: F711 공지사항, 액터(비회원/회원/관리자/외부) 정의
- API 확정: /api/interest-regions, /api/notices (코드 기준)
- WBS/간트에 시스템 다이어그램 작업(6.3) 추가, 다이어그램 참조 링크
- xlsx 재생성(F711·다이어그램 반영, 수식오류 0)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/deliverables/no-home-deliverables.xlsx
+++ b/docs/deliverables/no-home-deliverables.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1275,6 +1275,43 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>추가</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>F711</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>공지사항</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>공지 조회(전체)·관리(관리자 CRUD)</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>전효준</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>비회원 조회, 관리자만 CRUD</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1286,7 +1323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2645,30 +2682,67 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
+          <t>시스템 다이어그램(클래스·ERD·유스케이스)</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>공통</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>diagrams/</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>6.4</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
           <t>요구사항 명세서·WBS·간트</t>
         </is>
       </c>
-      <c r="C39" s="8" t="inlineStr">
+      <c r="C40" s="8" t="inlineStr">
         <is>
           <t>공통</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="E40" s="3" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="F40" s="3" t="inlineStr">
         <is>
           <t>진행중</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G40" s="3" t="inlineStr">
         <is>
           <t>deliverables/</t>
         </is>
@@ -2685,7 +2759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3367,7 +3441,7 @@
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>명세서·WBS·간트</t>
+          <t>시스템 다이어그램</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
@@ -3389,28 +3463,53 @@
       <c r="N27" s="12" t="n"/>
       <c r="O27" s="11" t="n"/>
     </row>
-    <row r="29">
-      <c r="A29" s="19" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>명세서·WBS·간트</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>공통</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="n"/>
+      <c r="D28" s="12" t="n"/>
+      <c r="E28" s="12" t="n"/>
+      <c r="F28" s="12" t="n"/>
+      <c r="G28" s="12" t="n"/>
+      <c r="H28" s="12" t="n"/>
+      <c r="I28" s="12" t="n"/>
+      <c r="J28" s="12" t="n"/>
+      <c r="K28" s="12" t="n"/>
+      <c r="L28" s="12" t="n"/>
+      <c r="M28" s="12" t="n"/>
+      <c r="N28" s="12" t="n"/>
+      <c r="O28" s="11" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="19" t="inlineStr">
         <is>
           <t>범례</t>
         </is>
       </c>
-      <c r="B29" s="20" t="inlineStr">
+      <c r="B30" s="20" t="inlineStr">
         <is>
           <t>이정헌</t>
         </is>
       </c>
-      <c r="C29" s="21" t="inlineStr">
+      <c r="C30" s="21" t="inlineStr">
         <is>
           <t>최민식</t>
         </is>
       </c>
-      <c r="D29" s="22" t="inlineStr">
+      <c r="D30" s="22" t="inlineStr">
         <is>
           <t>전효준</t>
         </is>
       </c>
-      <c r="E29" s="23" t="inlineStr">
+      <c r="E30" s="23" t="inlineStr">
         <is>
           <t>공통</t>
         </is>

</xml_diff>